<commit_message>
Task 2: BBT Testing - fully updated documentation
</commit_message>
<xml_diff>
--- a/Exam/gymtrackerpro/lib/__tests__/bbt/utils/escapeLike-bbt-form.xlsx
+++ b/Exam/gymtrackerpro/lib/__tests__/bbt/utils/escapeLike-bbt-form.xlsx
@@ -17,9 +17,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="126">
-  <si>
-    <t>Statement: escapeLike(s) – escapes the three LIKE meta-characters (%, _, \) so the result can be safely interpolated into a Prisma/SQL LIKE pattern. Used by findMembers, findAdmins, findAll exercises, and findAll workout-sessions when a search term is provided.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="102">
+  <si>
+    <t>Statement: escapeLike(s) – escapes the three LIKE meta-characters (%, _, \) so the result can be safely used in a Prisma/SQL LIKE pattern.</t>
   </si>
   <si>
     <t/>
@@ -37,7 +37,7 @@
     <t>precondition</t>
   </si>
   <si>
-    <t>None – pure function, no I/O</t>
+    <t>None</t>
   </si>
   <si>
     <t>Results</t>
@@ -70,6 +70,12 @@
     <t>returned unchanged</t>
   </si>
   <si>
+    <t>empty string</t>
+  </si>
+  <si>
+    <t>returns empty string</t>
+  </si>
+  <si>
     <t>% character present</t>
   </si>
   <si>
@@ -94,12 +100,6 @@
     <t>all specials escaped in order</t>
   </si>
   <si>
-    <t>empty string</t>
-  </si>
-  <si>
-    <t>returns empty string</t>
-  </si>
-  <si>
     <t>multiple consecutive % chars</t>
   </si>
   <si>
@@ -133,7 +133,7 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>1</t>
+    <t>EC-1</t>
   </si>
   <si>
     <t>"benchpress"</t>
@@ -142,7 +142,13 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>2</t>
+    <t>EC-2</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>EC-3</t>
   </si>
   <si>
     <t>"100%"</t>
@@ -151,7 +157,7 @@
     <t>"100\%"</t>
   </si>
   <si>
-    <t>3</t>
+    <t>EC-4</t>
   </si>
   <si>
     <t>"bench_press"</t>
@@ -160,7 +166,7 @@
     <t>"bench\_press"</t>
   </si>
   <si>
-    <t>4</t>
+    <t>EC-5</t>
   </si>
   <si>
     <t>"path\value"</t>
@@ -169,7 +175,7 @@
     <t>"path\\value"</t>
   </si>
   <si>
-    <t>5</t>
+    <t>EC-6</t>
   </si>
   <si>
     <t>"100%_bench\press"</t>
@@ -178,13 +184,7 @@
     <t>"100\%\_bench\\press"</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>""</t>
-  </si>
-  <si>
-    <t>7</t>
+    <t>EC-7</t>
   </si>
   <si>
     <t>"%%"</t>
@@ -193,7 +193,7 @@
     <t>"\%\%"</t>
   </si>
   <si>
-    <t>8</t>
+    <t>EC-8</t>
   </si>
   <si>
     <t>"__"</t>
@@ -202,7 +202,7 @@
     <t>"\_\_"</t>
   </si>
   <si>
-    <t>9</t>
+    <t>EC-9</t>
   </si>
   <si>
     <t>"\\"</t>
@@ -229,7 +229,7 @@
     <t>"a" (plain), "%" (percent), "_" (underscore), "\" (backslash)</t>
   </si>
   <si>
-    <t>n + 1 from minimum (n = 2)</t>
+    <t>n+1 from minimum (n = 2)</t>
   </si>
   <si>
     <t>"ab" (plain), "%%" (two percents), "__" (two underscores), "\\" (two backslashes)</t>
@@ -256,7 +256,7 @@
     <t>"_"</t>
   </si>
   <si>
-    <t>"\_ "</t>
+    <t>"\_"</t>
   </si>
   <si>
     <t>"\"</t>
@@ -274,87 +274,15 @@
     <t>TC from BVA</t>
   </si>
   <si>
-    <t>EC-1</t>
-  </si>
-  <si>
-    <t>"benchpress" (plain string)</t>
-  </si>
-  <si>
-    <t>EC-2</t>
-  </si>
-  <si>
-    <t>"100%" (percent)</t>
-  </si>
-  <si>
-    <t>EC-3</t>
-  </si>
-  <si>
-    <t>"bench_press" (underscore)</t>
-  </si>
-  <si>
-    <t>EC-4</t>
-  </si>
-  <si>
-    <t>"path\value" (backslash)</t>
-  </si>
-  <si>
-    <t>EC-5</t>
-  </si>
-  <si>
-    <t>"100%_bench\press" (mixed)</t>
-  </si>
-  <si>
-    <t>EC-6</t>
-  </si>
-  <si>
     <t>BVA-1</t>
   </si>
   <si>
-    <t>"" (empty, n=0)</t>
-  </si>
-  <si>
-    <t>EC-7</t>
+    <t>BVA-2</t>
   </si>
   <si>
     <t>BVA-3</t>
   </si>
   <si>
-    <t>"%%"  (consecutive %, n=2)</t>
-  </si>
-  <si>
-    <t>EC-8</t>
-  </si>
-  <si>
-    <t>"__"  (consecutive _, n=2)</t>
-  </si>
-  <si>
-    <t>EC-9</t>
-  </si>
-  <si>
-    <t>"\\" (consecutive \, n=2)</t>
-  </si>
-  <si>
-    <t>BVA-2</t>
-  </si>
-  <si>
-    <t>"a"   (plain char, n=1)</t>
-  </si>
-  <si>
-    <t>"%" (single %, n=1)</t>
-  </si>
-  <si>
-    <t>"_"  (single _, n=1)</t>
-  </si>
-  <si>
-    <t>"\_"</t>
-  </si>
-  <si>
-    <t>"\". (single \, n=1)</t>
-  </si>
-  <si>
-    <t>"ab"  (plain chars, n=2)</t>
-  </si>
-  <si>
     <t>Testing</t>
   </si>
   <si>
@@ -385,7 +313,7 @@
     <t>Re-tested</t>
   </si>
   <si>
-    <t>UTILS-ESCAPE</t>
+    <t>UTIL-01</t>
   </si>
   <si>
     <t>n/a</t>
@@ -1121,7 +1049,7 @@
         <v>42</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>40</v>
@@ -1132,13 +1060,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>40</v>
@@ -1149,13 +1077,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>40</v>
@@ -1166,13 +1094,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>40</v>
@@ -1183,10 +1111,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>54</v>
@@ -1349,10 +1277,10 @@
         <v>73</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>40</v>
@@ -1502,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1538,13 +1466,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>39</v>
@@ -1558,16 +1486,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>40</v>
@@ -1578,16 +1506,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>40</v>
@@ -1598,16 +1526,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>40</v>
@@ -1618,16 +1546,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>40</v>
@@ -1638,13 +1566,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>97</v>
+        <v>53</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>54</v>
@@ -1658,13 +1586,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>98</v>
+        <v>55</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>57</v>
@@ -1678,13 +1606,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>60</v>
@@ -1698,13 +1626,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>63</v>
@@ -1721,13 +1649,13 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>106</v>
+        <v>42</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>40</v>
@@ -1741,13 +1669,13 @@
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>40</v>
@@ -1761,13 +1689,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>108</v>
+        <v>76</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>40</v>
@@ -1781,13 +1709,13 @@
         <v>1</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>40</v>
@@ -1801,15 +1729,95 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>111</v>
+        <v>80</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="E16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1838,16 +1846,16 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
@@ -1855,45 +1863,45 @@
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>122</v>
+        <v>98</v>
       </c>
       <c r="B3" s="1">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D3" s="1">
         <v>0</v>
@@ -1902,19 +1910,19 @@
         <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="H3" s="1">
         <v>0</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>